<commit_message>
feat: add optativas endpoint to retrieve elective subjects for malla
The MallaController now exposes an `optativas` endpoint that returns
elective (optativa) subjects associated with a given malla curricular.
The endpoint:

- Resolves the optional slot context to label the optativa group.
- Fetches elective subjects from `programa_electivas` filtered by the
  malla's program.
- Ensures optativas are linked to the malla through a dedicated
  optativas grouping when missing.
- Includes prerequisite subjects and credit totals per optativa.
- Persists selected optativa slot assignments via `store` so the chosen
  subject is recorded in `agrupacion_asignatura` for the slot.

Supporting imports were added (Agrupacion, Componente, ProgramaElectiva,
Requisito) and a private helper was introduced to guarantee the optativa
grouping exists for the malla before returning data.
</commit_message>
<xml_diff>
--- a/files_tests/FORMATO DE CARGA - ADM. SISTEMAS.xlsx
+++ b/files_tests/FORMATO DE CARGA - ADM. SISTEMAS.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="34">
   <si>
     <t>Normativa</t>
   </si>
@@ -54,16 +54,13 @@
     <t>OPTATIVA2</t>
   </si>
   <si>
-    <t>Haber aprobado 100 crétidos (60%) del plan de estudios</t>
+    <t>Haber aprobado 100 créditos (60%) del plan de estudios</t>
   </si>
   <si>
     <t>Haber aprobado 24 créditos (29%) del componente profesional</t>
   </si>
   <si>
     <t xml:space="preserve">Haber aprobado 24 créditos (29%) del componente profesional </t>
-  </si>
-  <si>
-    <t>Haber aprobado 100 créditos (60%) del plan de estudios</t>
   </si>
   <si>
     <t>Haber aprobado 100 créditos (60%) del pna de estudios</t>
@@ -581,13 +578,13 @@
       <c r="A4" s="6">
         <v>7.0</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="1">
         <v>1.0</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="2">
         <v>17.0</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="2">
         <v>1000005.0</v>
       </c>
       <c r="E4" s="6" t="s">
@@ -1499,7 +1496,7 @@
         <v>9</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H40" s="6">
         <v>8.0</v>
@@ -1577,7 +1574,7 @@
         <v>9</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H43" s="6">
         <v>8.0</v>
@@ -1594,7 +1591,7 @@
         <v>25.0</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>11</v>
@@ -1616,7 +1613,7 @@
         <v>25.0</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>11</v>
@@ -1638,7 +1635,7 @@
         <v>25.0</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>11</v>
@@ -1669,7 +1666,7 @@
         <v>9</v>
       </c>
       <c r="G47" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H47" s="6">
         <v>10.0</v>
@@ -1721,7 +1718,7 @@
         <v>9</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H49" s="6">
         <v>10.0</v>
@@ -1738,7 +1735,7 @@
         <v>28.0</v>
       </c>
       <c r="D50" s="17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>11</v>
@@ -1760,7 +1757,7 @@
         <v>28.0</v>
       </c>
       <c r="D51" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>11</v>
@@ -1782,7 +1779,7 @@
         <v>28.0</v>
       </c>
       <c r="D52" s="17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>11</v>
@@ -1804,7 +1801,7 @@
         <v>28.0</v>
       </c>
       <c r="D53" s="17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>11</v>
@@ -1826,7 +1823,7 @@
         <v>28.0</v>
       </c>
       <c r="D54" s="17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>11</v>
@@ -1848,7 +1845,7 @@
         <v>28.0</v>
       </c>
       <c r="D55" s="17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>11</v>
@@ -1870,7 +1867,7 @@
         <v>28.0</v>
       </c>
       <c r="D56" s="17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>11</v>
@@ -1892,7 +1889,7 @@
         <v>28.0</v>
       </c>
       <c r="D57" s="17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>11</v>
@@ -1914,7 +1911,7 @@
         <v>28.0</v>
       </c>
       <c r="D58" s="17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>11</v>
@@ -1934,7 +1931,7 @@
         <v>28.0</v>
       </c>
       <c r="D59" s="17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>11</v>
@@ -1954,7 +1951,7 @@
         <v>28.0</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>11</v>
@@ -1974,7 +1971,7 @@
         <v>29.0</v>
       </c>
       <c r="D61" s="21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>11</v>
@@ -1994,7 +1991,7 @@
         <v>29.0</v>
       </c>
       <c r="D62" s="21" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
fix(api): permitir sufijos numéricos dinámicos en placeholders
Se actualiza la lógica de detección de placeholders en `ExcelParserService` para utilizar una expresión regular en lugar de una lista estática de códigos. Esto permite que códigos como 'OPTATIVA9', 'OPTATIVA10' o 'LIBRE12' sean reconocidos automáticamente como slots sin necesidad de modificar el código fuente cuando se añaden más elementos en el Excel.

Además, se realizan ajustes en el frontend para mejorar la gestión de estados de carga y limpieza de diálogos de confirmación en el componente de asignación de optativas.

Se añaden pruebas unitarias para verificar la detección de nuevos sufijos y asegurar que se procesen correctamente como slots.
</commit_message>
<xml_diff>
--- a/files_tests/FORMATO DE CARGA - ADM. SISTEMAS.xlsx
+++ b/files_tests/FORMATO DE CARGA - ADM. SISTEMAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Escritorio\Proyecto_Mallas\mallas\files_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F3679C6-9D07-457F-A20F-A7EC7094D9F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6159DF28-03D9-4A54-AF75-2878AB7F4CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="37">
   <si>
     <t>Normativa</t>
   </si>
@@ -125,6 +125,15 @@
   </si>
   <si>
     <t>NIVELATORIO 2</t>
+  </si>
+  <si>
+    <t>OPTATIVA8</t>
+  </si>
+  <si>
+    <t>OPTATIVA9</t>
+  </si>
+  <si>
+    <t>OPTATIVA10</t>
   </si>
 </sst>
 </file>
@@ -2129,25 +2138,70 @@
       </c>
     </row>
     <row r="67" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="D67" s="18"/>
-      <c r="E67" s="18"/>
-      <c r="F67" s="18"/>
-      <c r="G67" s="18"/>
-      <c r="H67" s="18"/>
+      <c r="A67" s="16">
+        <v>7</v>
+      </c>
+      <c r="B67" s="16">
+        <v>2</v>
+      </c>
+      <c r="C67" s="7">
+        <v>25</v>
+      </c>
+      <c r="D67" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E67" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F67" s="7"/>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7">
+        <v>7</v>
+      </c>
     </row>
     <row r="68" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="D68" s="18"/>
-      <c r="E68" s="18"/>
-      <c r="F68" s="18"/>
-      <c r="G68" s="18"/>
-      <c r="H68" s="18"/>
+      <c r="A68" s="16">
+        <v>7</v>
+      </c>
+      <c r="B68" s="16">
+        <v>2</v>
+      </c>
+      <c r="C68" s="7">
+        <v>25</v>
+      </c>
+      <c r="D68" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F68" s="7"/>
+      <c r="G68" s="7"/>
+      <c r="H68" s="7">
+        <v>4</v>
+      </c>
     </row>
     <row r="69" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="D69" s="18"/>
-      <c r="E69" s="18"/>
-      <c r="F69" s="18"/>
-      <c r="G69" s="18"/>
-      <c r="H69" s="18"/>
+      <c r="A69" s="16">
+        <v>7</v>
+      </c>
+      <c r="B69" s="16">
+        <v>2</v>
+      </c>
+      <c r="C69" s="7">
+        <v>25</v>
+      </c>
+      <c r="D69" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F69" s="7"/>
+      <c r="G69" s="7"/>
+      <c r="H69" s="7">
+        <v>8</v>
+      </c>
     </row>
     <row r="70" spans="1:8" ht="12.75" x14ac:dyDescent="0.2">
       <c r="D70" s="18"/>
@@ -8648,7 +8702,7 @@
   </sheetData>
   <autoFilter ref="A1:Z997" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E66" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E66 E67:E69" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>